<commit_message>
test: add test cases for occupancyInfoList
</commit_message>
<xml_diff>
--- a/__fixtures__/simple-multisheet.xlsx
+++ b/__fixtures__/simple-multisheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kendrick/Documents/git/community-db/__fixtures__/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75F9D662-6126-6B4F-B41E-E242B28E7CB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7C2A49E-6EE0-DC47-B36E-AAC76D187E01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1660" yWindow="600" windowWidth="49540" windowHeight="28200" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1720" yWindow="600" windowWidth="49480" windowHeight="28200" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Community" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="103">
   <si>
     <t>name</t>
   </si>
@@ -323,19 +323,36 @@
   </si>
   <si>
     <t>Sample Community</t>
+  </si>
+  <si>
+    <t>Previous</t>
+  </si>
+  <si>
+    <t>Owner</t>
+  </si>
+  <si>
+    <t>2010-01-01T00:00:00.000Z</t>
+  </si>
+  <si>
+    <t>2015-02-01T00:00:00.000Z</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF11181C"/>
+      <name val="Inter"/>
     </font>
   </fonts>
   <fills count="2">
@@ -358,8 +375,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -700,9 +718,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -731,7 +749,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:9">
       <c r="A2" t="s">
         <v>98</v>
       </c>
@@ -765,9 +783,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:L3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12">
       <c r="A1" t="s">
         <v>15</v>
       </c>
@@ -805,7 +823,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:12">
       <c r="A2">
         <v>1</v>
       </c>
@@ -831,7 +849,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:12">
       <c r="A3">
         <v>2</v>
       </c>
@@ -864,10 +882,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:H5"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:H6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8">
       <c r="A1" t="s">
         <v>34</v>
       </c>
@@ -893,7 +911,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8">
       <c r="A2">
         <v>1</v>
       </c>
@@ -916,7 +934,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8">
       <c r="A3">
         <v>2</v>
       </c>
@@ -939,7 +957,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8">
       <c r="A4">
         <v>3</v>
       </c>
@@ -962,7 +980,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8">
       <c r="A5">
         <v>4</v>
       </c>
@@ -980,6 +998,29 @@
       </c>
       <c r="H5" t="s">
         <v>43</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="18">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6" t="s">
+        <v>99</v>
+      </c>
+      <c r="E6" t="s">
+        <v>100</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>102</v>
       </c>
     </row>
   </sheetData>
@@ -993,9 +1034,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:E9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5">
       <c r="A1" t="s">
         <v>50</v>
       </c>
@@ -1012,7 +1053,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1029,7 +1070,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1046,7 +1087,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1063,7 +1104,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1080,7 +1121,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:5">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1097,7 +1138,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:5">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1114,7 +1155,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:5">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1131,7 +1172,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:5">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1159,9 +1200,9 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:G9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7">
       <c r="A1" t="s">
         <v>68</v>
       </c>
@@ -1184,7 +1225,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1201,7 +1242,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1224,7 +1265,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1238,7 +1279,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1255,7 +1296,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1272,7 +1313,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1295,7 +1336,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1315,7 +1356,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1346,9 +1387,9 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:D6"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4">
       <c r="A1" t="s">
         <v>79</v>
       </c>
@@ -1362,7 +1403,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1376,7 +1417,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1390,7 +1431,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1404,7 +1445,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1418,7 +1459,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1444,9 +1485,9 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:F7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6">
       <c r="A1" t="s">
         <v>89</v>
       </c>
@@ -1466,7 +1507,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1486,7 +1527,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1506,7 +1547,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1526,7 +1567,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1546,7 +1587,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1566,7 +1607,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6">
       <c r="A7">
         <v>6</v>
       </c>

</xml_diff>

<commit_message>
fix: add background when autocomplete is active (#309)
</commit_message>
<xml_diff>
--- a/__fixtures__/simple-multisheet.xlsx
+++ b/__fixtures__/simple-multisheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kendrick/Documents/git/community-db/__fixtures__/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75F9D662-6126-6B4F-B41E-E242B28E7CB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7C2A49E-6EE0-DC47-B36E-AAC76D187E01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1660" yWindow="600" windowWidth="49540" windowHeight="28200" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1720" yWindow="600" windowWidth="49480" windowHeight="28200" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Community" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="103">
   <si>
     <t>name</t>
   </si>
@@ -323,19 +323,36 @@
   </si>
   <si>
     <t>Sample Community</t>
+  </si>
+  <si>
+    <t>Previous</t>
+  </si>
+  <si>
+    <t>Owner</t>
+  </si>
+  <si>
+    <t>2010-01-01T00:00:00.000Z</t>
+  </si>
+  <si>
+    <t>2015-02-01T00:00:00.000Z</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color rgb="FF11181C"/>
+      <name val="Inter"/>
     </font>
   </fonts>
   <fills count="2">
@@ -358,8 +375,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -700,9 +718,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -731,7 +749,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:9">
       <c r="A2" t="s">
         <v>98</v>
       </c>
@@ -765,9 +783,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:L3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12">
       <c r="A1" t="s">
         <v>15</v>
       </c>
@@ -805,7 +823,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:12">
       <c r="A2">
         <v>1</v>
       </c>
@@ -831,7 +849,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:12">
       <c r="A3">
         <v>2</v>
       </c>
@@ -864,10 +882,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:H5"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:H6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8">
       <c r="A1" t="s">
         <v>34</v>
       </c>
@@ -893,7 +911,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8">
       <c r="A2">
         <v>1</v>
       </c>
@@ -916,7 +934,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:8">
       <c r="A3">
         <v>2</v>
       </c>
@@ -939,7 +957,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:8">
       <c r="A4">
         <v>3</v>
       </c>
@@ -962,7 +980,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:8">
       <c r="A5">
         <v>4</v>
       </c>
@@ -980,6 +998,29 @@
       </c>
       <c r="H5" t="s">
         <v>43</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="18">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6">
+        <v>1</v>
+      </c>
+      <c r="D6" t="s">
+        <v>99</v>
+      </c>
+      <c r="E6" t="s">
+        <v>100</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>102</v>
       </c>
     </row>
   </sheetData>
@@ -993,9 +1034,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:E9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5">
       <c r="A1" t="s">
         <v>50</v>
       </c>
@@ -1012,7 +1053,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1029,7 +1070,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1046,7 +1087,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1063,7 +1104,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1080,7 +1121,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:5">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1097,7 +1138,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:5">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1114,7 +1155,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:5">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1131,7 +1172,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:5">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1159,9 +1200,9 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:G9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7">
       <c r="A1" t="s">
         <v>68</v>
       </c>
@@ -1184,7 +1225,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1201,7 +1242,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1224,7 +1265,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1238,7 +1279,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1255,7 +1296,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1272,7 +1313,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7">
       <c r="A7">
         <v>6</v>
       </c>
@@ -1295,7 +1336,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7">
       <c r="A8">
         <v>7</v>
       </c>
@@ -1315,7 +1356,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7">
       <c r="A9">
         <v>8</v>
       </c>
@@ -1346,9 +1387,9 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:D6"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4">
       <c r="A1" t="s">
         <v>79</v>
       </c>
@@ -1362,7 +1403,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1376,7 +1417,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1390,7 +1431,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1404,7 +1445,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1418,7 +1459,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1444,9 +1485,9 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:F7"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6">
       <c r="A1" t="s">
         <v>89</v>
       </c>
@@ -1466,7 +1507,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6">
       <c r="A2">
         <v>1</v>
       </c>
@@ -1486,7 +1527,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6">
       <c r="A3">
         <v>2</v>
       </c>
@@ -1506,7 +1547,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6">
       <c r="A4">
         <v>3</v>
       </c>
@@ -1526,7 +1567,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6">
       <c r="A5">
         <v>4</v>
       </c>
@@ -1546,7 +1587,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6">
       <c r="A6">
         <v>5</v>
       </c>
@@ -1566,7 +1607,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6">
       <c r="A7">
         <v>6</v>
       </c>

</xml_diff>